<commit_message>
Pilot forecast: Hosts needed sensitivity sheet (Main follow-up to C1)
Steady weekly reconnected members for 12 to 80 Table Hosts, hosting
fortnightly or weekly, at 6 or 8 seats a table, with the fill and other
levers in blue; cells at or above the 60-a-week target turn green.
Prototype inputs; 184 formulas, no errors after recalc.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/research/pilot-forecast.xlsx
+++ b/design/research/pilot-forecast.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Weekly" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Funnel" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Targets vs live" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Hosts needed" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -105,7 +106,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="128">
   <si>
     <t xml:space="preserve">PROTOTYPE INPUTS, NOT DATA. Every blue number is an assumption to replace with real pilot figures. Nothing here is a measured result.</t>
   </si>
@@ -459,6 +460,36 @@
   </si>
   <si>
     <t xml:space="preserve">Reads: at today's assumptions, seats run out from week 4, so supply (hosts and tables), not sign-ups, limits the north star.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosts needed: week-8 reconnected members for hosts × tables per fortnight × seats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each cell: steady weekly reconnected = seats a week × fill × RSVP→check-in × repeat share × 'sits with someone met before'. Change the blue levers; cells at or above the target turn green.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fill assumed (sold-out tables are capped at 100%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repeat share of RSVPs (from Weekly, week 8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target: reconnected a week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other tables a week (not host-run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seats per table = 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table Hosts ↓ / tables per host per fortnight →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seats per table = 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 table per fortnight = today's Regular Table rhythm; 2 = every host runs a table every week. Hosts here replace the Weekly sheet's host build-up: this is a steady week, not week 8 of a ramp.</t>
   </si>
 </sst>
 </file>
@@ -625,7 +656,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -711,6 +742,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2459,4 +2510,361 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="22" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="23" t="n">
+        <f aca="false">IF(Weekly!I12=0,0,Weekly!H12/Weekly!I12)</f>
+        <v>0.739317293332755</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="24" t="n">
+        <f aca="false">'Targets vs live'!B6</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="24" t="n">
+        <f aca="false">Assumptions!$B$11</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="B11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" s="14" t="n">
+        <f aca="false">($A12*B$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>18.4444878340656</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <f aca="false">($A12*C$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>27.6667317510983</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="B13" s="14" t="n">
+        <f aca="false">($A13*B$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>21.5185691397432</v>
+      </c>
+      <c r="C13" s="14" t="n">
+        <f aca="false">($A13*C$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>33.8148943624535</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B14" s="14" t="n">
+        <f aca="false">($A14*B$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>27.6667317510983</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <f aca="false">($A14*C$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>46.1112195851639</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="B15" s="14" t="n">
+        <f aca="false">($A15*B$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>33.8148943624535</v>
+      </c>
+      <c r="C15" s="14" t="n">
+        <f aca="false">($A15*C$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>58.4075448078743</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="25" t="n">
+        <v>48</v>
+      </c>
+      <c r="B16" s="14" t="n">
+        <f aca="false">($A16*B$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>46.1112195851639</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <f aca="false">($A16*C$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>83.000195253295</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="25" t="n">
+        <v>64</v>
+      </c>
+      <c r="B17" s="14" t="n">
+        <f aca="false">($A17*B$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>58.4075448078743</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <f aca="false">($A17*C$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>107.592845698716</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="25" t="n">
+        <v>80</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <f aca="false">($A18*B$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>70.7038700305847</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <f aca="false">($A18*C$11/2+$B$8)*$B$10*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>132.185496144137</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B20" s="25" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="B21" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B22" s="14" t="n">
+        <f aca="false">($A22*B$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>24.5926504454207</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <f aca="false">($A22*C$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>36.8889756681311</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="14" t="n">
+        <f aca="false">($A23*B$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>28.6914255196575</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <f aca="false">($A23*C$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>45.0865258166047</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <f aca="false">($A24*B$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>36.8889756681311</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <f aca="false">($A24*C$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>61.4816261135519</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="B25" s="14" t="n">
+        <f aca="false">($A25*B$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>45.0865258166047</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <f aca="false">($A25*C$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>77.8767264104991</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="25" t="n">
+        <v>48</v>
+      </c>
+      <c r="B26" s="14" t="n">
+        <f aca="false">($A26*B$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>61.4816261135519</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <f aca="false">($A26*C$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>110.666927004393</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="25" t="n">
+        <v>64</v>
+      </c>
+      <c r="B27" s="14" t="n">
+        <f aca="false">($A27*B$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>77.8767264104991</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <f aca="false">($A27*C$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>143.457127598288</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="25" t="n">
+        <v>80</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <f aca="false">($A28*B$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>94.2718267074462</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <f aca="false">($A28*C$21/2+$B$8)*$B$20*MIN(1,$B$5)*Assumptions!$B$19*$B$6*Assumptions!$B$20</f>
+        <v>176.247328192182</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B12:C18">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B12&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B12&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B12&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B12&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B12&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B12&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B12&gt;=$B$7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B22:C28">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B22&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B22&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B22&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B22&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B22&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B22&gt;=$B$7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>B22&gt;=$B$7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>